<commit_message>
Offer assisted import for NOK 150 on the import page and in the template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TyRR9TLskkUJVdEZy8vSuG
</commit_message>
<xml_diff>
--- a/public/import-template-allseats.xlsx
+++ b/public/import-template-allseats.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,12 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F6B4F"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -101,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -127,6 +133,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -832,7 +841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D27"/>
+  <dimension ref="A2:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1155,8 +1164,19 @@
       <c r="C27" s="12" t="n"/>
       <c r="D27" s="12" t="n"/>
     </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Would you rather we did it? Send the file to post@allseats.no and we'll import the contacts for you for NOK 150 excl. VAT.</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C10:D10"/>

</xml_diff>